<commit_message>
Refresh the client work-hours statement generator and exports.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/CleverSolutions-Work-Hours-Statement-client.xlsx
+++ b/docs/CleverSolutions-Work-Hours-Statement-client.xlsx
@@ -12,7 +12,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -70,7 +70,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09 — 2026-08-11 (3 days)</t>
         </is>
       </c>
     </row>
@@ -129,42 +129,66 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16.25</v>
+        <v>20.0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Client hour envelope</t>
+          <t>Day 1 — 09.08.2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Quoted / promised range: 20–30 hours total for the engagement</t>
+          <t>6.5 h — project setup, content system, data layer, design tokens</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Remaining buffer (approx.)</t>
+          <t>Day 2 — 10.08.2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>~3.75–13.75 hours left for product data import, images, QA (depends on final quote 20 vs 30)</t>
+          <t>7.0 h — pages, navigation, contact API, SEO, smoke tests</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Day 3 — 11.08.2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>6.5 h — upgrade, brand polish, navbar motion, DriftWall backgrounds, handoff</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Remaining scope (approx.)</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>~0–10 h buffer within 20–30 h quote for bulk product import (150–180 SKUs) and images</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Currency note</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Hours halved vs internal build log to match the 20–30h client promise; use for pay orientation, not calendar time</t>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Hours are task-based estimates for client billing orientation; adjust rate as agreed</t>
         </is>
       </c>
     </row>
@@ -174,7 +198,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -224,7 +248,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -234,25 +258,25 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Read rebuild brief; scaffold Next.js App Router project with TypeScript, Tailwind, ESLint, project conventions</t>
+          <t>Read rebuild brief; scaffold Next.js App Router project with TypeScript, Tailwind, ESLint</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Empty workspace; need production-ready base aligned to brief (gallery not store)</t>
+          <t>Empty workspace; gallery site (not store); production-ready foundation needed</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Scaffolded Next.js app; configured path aliases, Tailwind tokens, fonts (display + sans with Cyrillic), base layout shell</t>
+          <t>Scaffolded app; path aliases, Tailwind tokens, Cyrillic fonts, base layout, AGENTS conventions</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>package.json, app/, tailwind.config.ts, AGENTS.md conventions</t>
+          <t>package.json, app/, tailwind.config.ts, AGENTS.md</t>
         </is>
       </c>
     </row>
@@ -262,7 +286,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -277,16 +301,16 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>UI must be bg-BG; editors need one place for copy</t>
+          <t>UI must be bg-BG; single editable copy source for non-developer updates</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Centralized content/bg.ts with site, nav, hero, categories, product, contact, footer strings</t>
+          <t>Centralized content/bg.ts for site, nav, hero, categories, product, contact, footer</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>0.75</v>
+        <v>1.0</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -300,7 +324,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -315,20 +339,20 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>No CMS; real data arrives later from paper records; must avoid schema churn</t>
+          <t>No CMS; real data from paper records later; schema must stay stable</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>ProductSchema + per-category TS files; draft vs published; optional priceBgn; empty images = placeholder; index helpers</t>
+          <t>ProductSchema; per-category files; draft/published; optional price; index helpers</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>1.5</v>
+        <v>1.75</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>data/products/{schema,index,kitchenware,security,wristbands,vacuums}.ts</t>
+          <t>data/products/*</t>
         </is>
       </c>
     </row>
@@ -338,7 +362,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -348,25 +372,25 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Visual system: tokens, typography, skeletons, motion primitives</t>
+          <t>Tokens, typography, skeletons, SSR-safe motion primitives</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Need maintainable UI; loading states must match layout; SSR motion pitfalls</t>
+          <t>Loading states must match layouts; Framer SSR blank-page risk</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Canvas/ink tokens; skeleton shimmer; ScrollReveal with SSR-safe mount (avoid opacity:0 blank page)</t>
+          <t>Ink/canvas tokens; skeleton shimmer; ScrollReveal safe mount pattern</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>1.0</v>
+        <v>1.75</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>app/globals.css, components/skeletons, components/motion</t>
+          <t>globals.css, components/skeletons, components/motion</t>
         </is>
       </c>
     </row>
@@ -386,21 +410,21 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Header/Footer with category nav, mobile menu, subcategory dropdowns</t>
+          <t>Header/Footer; category nav; mobile menu; subcategory dropdowns</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Four unrelated categories need clear IA; English routes for URLs, BG labels</t>
+          <t>Four categories; English URL slugs with Bulgarian labels</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Sticky header, hover dropdowns with English query slugs, responsive drawer menu, footer links + contact</t>
+          <t>Sticky header, hover dropdowns, responsive drawer, footer structure</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>1.0</v>
+        <v>1.25</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -424,25 +448,25 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Hero + category grid + featured products + contact CTA</t>
+          <t>Hero, category grid, featured products, contact CTA block</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Brand-first hero with real product photography (not stock collage)</t>
+          <t>Brand-first hero with local product photography</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Hero10 fan of local hero images; HomeSections for categories/featured/contact; primary CTAs</t>
+          <t>Hero10 image fan; HomeSections; primary/secondary CTAs</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>1.25</v>
+        <v>1.5</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>components/home/*, components/ui/hero-10.tsx, app/page.tsx, public/images/hero</t>
+          <t>components/home/*, components/ui/hero-10.tsx, app/page.tsx</t>
         </is>
       </c>
     </row>
@@ -457,30 +481,30 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Category pages</t>
+          <t>Category &amp; product pages</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Kitchen / Security / Wristbands / Vacuums galleries + empty/coming-soon states</t>
+          <t>Galleries, coming-soon states, product detail with gallery/specs/JSON-LD</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Some categories sparse; drafts must stay hidden</t>
+          <t>SEO without checkout; async App Router params on Next 16</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Shared CategoryPageContent; ComingSoon state; product grids filtered to published only</t>
+          <t>CategoryPageContent; ProductGallery/Specs; generateStaticParams; contact deep-link</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>1.0</v>
+        <v>1.75</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>app/{kitchen,security,wristbands,vacuums}, lib/category-page.tsx</t>
+          <t>app/{kitchen,security,wristbands,vacuums}, app/product/[slug]/*</t>
         </is>
       </c>
     </row>
@@ -495,22 +519,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Product detail</t>
+          <t>Contact &amp; email</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Product page: gallery, specs, description, JSON-LD, contact deep-link</t>
+          <t>Contact page + Resend API Route Handler</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SEO + conversion without checkout; async params on modern Next</t>
+          <t>Production email path with env-based configuration</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Dynamic /product/[slug]; generateStaticParams; metadata; gallery/specs; contact?product=; Product JSON-LD</t>
+          <t>Validated form; POST /api/contact; .env.example</t>
         </is>
       </c>
       <c r="G9" t="n">
@@ -518,7 +542,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>app/product/[slug]/*, components/products/*, lib/product-jsonld.ts</t>
+          <t>app/contact, components/contact/ContactForm.tsx, app/api/contact</t>
         </is>
       </c>
     </row>
@@ -533,30 +557,30 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Contact &amp; email</t>
+          <t>Assets, SEO &amp; QA</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Contact page + API Route Handler with Resend</t>
+          <t>Local images, metadata/sitemap, Playwright smoke tests</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Need production email path with env-based config</t>
+          <t>No remote stock dependency; regression safety before handoff</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Validated form UI; POST /api/contact; .env.example for RESEND_* and site URL</t>
+          <t>public/images/*; robots/sitemap; e2e smoke suite (14 paths)</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>1.0</v>
+        <v>1.25</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>app/contact, components/contact/ContactForm.tsx, app/api/contact, .env.example</t>
+          <t>public/images, SEO files, e2e/smoke.spec.ts</t>
         </is>
       </c>
     </row>
@@ -566,35 +590,35 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Media &amp; assets</t>
+          <t>Platform upgrade</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Local image pipeline for hero and kitchen sample products</t>
+          <t>Upgrade to Next.js 16 and React 19; fix breaking changes</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Avoid remote Unsplash dependency; empty image arrays must degrade gracefully</t>
+          <t>Codemod hung; params Promise migration; build verification</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>public/images structure; ImagePlaceholder; Next Image usage</t>
+          <t>Manual dep upgrade; async params fixes; verified production build</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>public/images/products/sample-*, ImagePlaceholder.tsx</t>
+          <t>package.json, product page params, eslint-config-next 16</t>
         </is>
       </c>
     </row>
@@ -604,35 +628,35 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Routing &amp; SEO</t>
+          <t>Brand &amp; UX polish</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>English public routes; sitemap/robots/metadata; remove Cyrillic URL friction</t>
+          <t>Teal accent, scrollbar, product card Details flow, scroll-to-top, footer credit</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Cyrillic/Latin slug confusion; need stable English paths with BG UI</t>
+          <t>Monochrome UI; cards pushed contact too early; mobile polish</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Routes: /, /kitchen, /security, /wristbands, /vacuums, /product/[slug], /contact; metadata + SEO files</t>
+          <t>brand tokens; ProductCard Details CTA; ScrollToTop; subtle NRG footer link</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>app routes, lib/site-config.ts, SEO files</t>
+          <t>globals.css, tailwind.config.ts, ProductCard, ScrollToTop, Footer</t>
         </is>
       </c>
     </row>
@@ -642,35 +666,35 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>QA automation</t>
+          <t>Navbar motion</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Playwright smoke tests for critical paths</t>
+          <t>Port NRGxPortfolio scroll-shrink navbar behaviour</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Need regression safety for gallery + contact flows</t>
+          <t>Client wanted same motion language as portfolio site</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>e2e smoke suite (home, categories, product, contact, draft hidden); playwright config</t>
+          <t>Scroll-shrink pill header, cursor sheen, underline hovers, animated mobile menu</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0.75</v>
+        <v>1.0</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>e2e/smoke.spec.ts, playwright.config.ts</t>
+          <t>components/layout/Header.tsx</t>
         </is>
       </c>
     </row>
@@ -680,35 +704,35 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Platform upgrade</t>
+          <t>Homepage backgrounds</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Upgrade Next.js 14 to 16 and React 19; fix breaking changes</t>
+          <t>DriftWall full-page backdrop; layered category/contact panels; inner-page teal gradient</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Interactive codemod hung; App Router async params; dependency engine warnings</t>
+          <t>Hero atmosphere vs readable content sections; footer above fixed background</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Manual dependency bump; params Promise fixes; Vercel plugin guidance; verified build</t>
+          <t>DriftWall + HomePageBackground; MainBackground route switch; PageGradientBackground</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>1.25</v>
+        <v>1.75</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>package.json, product page params, eslint-config-next 16</t>
+          <t>DriftWall.jsx, HomePageBackground, PageGradientBackground, HomeSections</t>
         </is>
       </c>
     </row>
@@ -718,27 +742,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>DevOps / DX</t>
+          <t>Bugfixes &amp; DX</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Fix Windows .next lock/corruption and blank-page SSR motion issues</t>
+          <t>React 19 script warning, Windows .next cache, JSON-LD, dev scripts</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Dev server hung on Starting; corrupted .next; Framer opacity:0 hid content</t>
+          <t>Balancer script tag; dev server lock; console warnings</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>npm run clean / dev:fresh scripts; ScrollReveal mounts plain div until client ready</t>
+          <t>Removed react-wrap-balancer; clean/dev:fresh; data-scroll-behavior; JSON-LD pattern</t>
         </is>
       </c>
       <c r="G15" t="n">
@@ -746,7 +770,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>package.json scripts, ScrollReveal.tsx</t>
+          <t>hero-10.tsx, package.json scripts, app/layout.tsx</t>
         </is>
       </c>
     </row>
@@ -756,149 +780,35 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>UX iteration</t>
+          <t>Client handoff prep</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Product cards: brief info + full-width Details CTA; equal-height cards</t>
+          <t>Product Excel import template; hours statement; git push to GitHub</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Cards previously over-emphasized contact; need browse then detail flow</t>
+          <t>Client needs format for 150–180 products; billing documentation</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Details CTA; mt-auto pinned button; grid items-stretch; contact CTA only on detail</t>
+          <t>CleverSolutions-Produktov-shablon.xlsx; work-hours statement; commits on main</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>ProductCard.tsx, ProductGrid.tsx, skeletons, content/bg.ts</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="n">
-        <v>16.0</v>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>Brand &amp; polish</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Site teal accent + custom scrollbar matching brand</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>Default OS scrollbar + grey-only UI felt unfinished</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>brand tokens in Tailwind/CSS; primary/CTAs/header/footer; scrollbar WebKit + Firefox; selection/focus</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>globals.css, tailwind.config.ts, lib/utils.ts, Header/Footer/CTAs</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="n">
-        <v>17.0</v>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>Bugfix</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>React 19 console error: script tag while rendering (hero)</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>react-wrap-balancer injects script; React 19 forbids that client path</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>Removed Balancer; CSS text-balance; uninstalled dependency; data-scroll-behavior on html</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>hero-10.tsx, app/layout.tsx, package.json</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="n">
-        <v>18.0</v>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>2026-08-10</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Handoff</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>Git commits, GitHub push, documentation of hours for reporting</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Need auditable history + hours justification artifact</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>Committed/pushed main; produced this Excel work statement</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>git history, docs/CleverSolutions-Work-Hours-Statement.xlsx</t>
+          <t>docs/*, scripts/generate-product-template.py, GitHub main branch</t>
         </is>
       </c>
     </row>
@@ -908,7 +818,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1188,20 +1098,47 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Monochrome UI lacked brand identity</t>
+          <t>DriftWall background readability on homepage</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Site felt generic</t>
+          <t>Featured heading hard to read over dark tiles</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Teal brand accent + branded scrollbar/selection/CTAs</t>
+          <t>Frosted panel on featured header; layered section backgrounds</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>P11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Inner-page teal gradient too strong then invisible</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Background tuning iterations</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Top-down softer wash with visible but non-aggressive teal</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -1319,7 +1256,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>910e54c initial site · a38c483 Next 16 upgrade · follow-up commit brand/UX/bugfixes + this statement</t>
+          <t>910e54c initial site · a38c483 Next 16 · brand/UX · navbar motion · f5af12d DriftWall backgrounds</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill DriftWall columns to the viewport and refresh work-hours exports.
Grow backdrop columns on wide screens so the floating image wall covers empty side space, and include the latest client work-hours statement updates.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/CleverSolutions-Work-Hours-Statement-client.xlsx
+++ b/docs/CleverSolutions-Work-Hours-Statement-client.xlsx
@@ -6,13 +6,14 @@
     <sheet name="Hours Log" sheetId="2" r:id="rId2"/>
     <sheet name="Problems Solutions" sheetId="3" r:id="rId3"/>
     <sheet name="Deliverables" sheetId="4" r:id="rId4"/>
+    <sheet name="Remaining SKUs" sheetId="5" r:id="rId5"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -70,7 +71,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-08-09 — 2026-08-11 (3 days)</t>
+          <t>2026-08-09 — 2026-08-23 (site build + catalogue + brand round)</t>
         </is>
       </c>
     </row>
@@ -129,7 +130,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>20.0</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="11">
@@ -171,22 +172,82 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Remaining scope (approx.)</t>
+          <t>Day 4 — 20.08.2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>~0–10 h buffer within 20–30 h quote for bulk product import (150–180 SKUs) and images</t>
+          <t>5.0 h — kitchen catalogue Excel import (39 SKUs + images)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Day 5 — 21.08.2026</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>0.75 h — catalogue text cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Day 6 — 22.08.2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>3.5 h — orange brand, logo/favicon, bilingual About page</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Day 7 — 23.08.2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2.25 h — hero category links, product image fit, hours statement</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Live catalogue now</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>39 real kitchen SKUs published; 12 sample placeholders in other categories (to replace)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Remaining products (ballpark)</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>150–180 SKUs still to enter: likely 24–36 h if Excel+images match the kitchen catalogue; 40–50 h if copy/images need heavy cleanup</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Currency note</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Hours are task-based estimates for client billing orientation; adjust rate as agreed</t>
         </is>
@@ -198,7 +259,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H21"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -809,6 +870,196 @@
       <c r="H16" t="inlineStr">
         <is>
           <t>docs/*, scripts/generate-product-template.py, GitHub main branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>16.0</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Catalogue import</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Import kitchen equipment Excel into published products with images</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>150–180 SKU catalogue; first real data was a multi-sheet Excel with embedded photos</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>import-catalogue.py: sheet→subcategory map, image extract, slugify, Zod-ready kitchenware.ts</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>scripts/import-catalogue.py, data/products/kitchenware.ts, public/images/products/*</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17.0</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Catalogue QA</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Normalize imported catalogue text endings and incomplete punctuation</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Excel cells had truncated sentences and inconsistent spacing</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Cleaned descriptions/specs in kitchenware.ts without changing product count</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>data/products/kitchenware.ts</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18.0</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-08-22</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Brand &amp; About</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Orange/black palette, logo mark favicon, bilingual За нас page</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Client asked for About copy, warmer color, logo colors black+orange</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Brand tokens #FF6000; BrandLogo; /about BG+EN; nav/footer; icon/apple-icon/favicon</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>content/bg.ts, app/about, BrandLogo, globals.css, app/icon.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19.0</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Homepage &amp; product photos</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Hero fan links to categories; 7-column DriftWall; contain product images</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Carousel photos needed to be category buttons; SKU photos cropped out of frames</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Clickable hero slides; column-grouped DriftWall; object-contain on cards/gallery</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>1.75</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>Hero.tsx, hero-10.tsx, hero-drift-images.ts, ProductCard, ProductGallery</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20.0</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Billing estimate</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Update work-hours statement and remaining 150–180 SKU ballpark</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Client needs hours-to-date plus time to finish remaining products</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Extended hours log to 31.5 h; Remaining SKUs sheet with scenario ranges</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>scripts/generate-work-statement.py, docs/CleverSolutions-Work-Hours-Statement-client.*</t>
         </is>
       </c>
     </row>
@@ -818,7 +1069,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -1135,12 +1386,93 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Top-down softer wash with visible but non-aggressive teal</t>
+          <t>Top-down softer wash; later replaced with warm orange from logo</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>P12</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Product photos overflowed frames / not centered</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Catalogue images cropped on cards and detail gallery</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>object-contain + padding on ProductCard and ProductGallery</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>P13</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Missing За нас and teal palette vs logo</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>No About page; brand colors did not match black/orange logo</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Bilingual /about; #FF6000 tokens; logo + C-mark favicon</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Resolved</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>P14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Remaining 150–180 SKUs not yet on the site</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Only 39 real kitchen products live; other categories are samples</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Kitchen importer exists; other categories need the same Excel+images package</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Open — see Remaining SKUs sheet</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1504,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>/ · /kitchen · /security · /wristbands · /vacuums · /product/[slug] · /contact</t>
+          <t>/ · /about · /kitchen · /security · /wristbands · /vacuums · /product/[slug] · /contact</t>
         </is>
       </c>
     </row>
@@ -1196,7 +1528,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Zod Product schema; 4 category datasets; published/draft; optional price &amp; buyUrl</t>
+          <t>Zod Product schema; 39 published kitchen SKUs from Excel; sample placeholders in 3 other categories</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1588,179 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>910e54c initial site · a38c483 Next 16 · brand/UX · navbar motion · f5af12d DriftWall backgrounds</t>
+          <t>910e54c initial site · 4c816f6 kitchen catalogue · e0cd666 brand/About · 436eeae hero links + image fit</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F6"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>SKU count</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Input quality</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Hours low</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Hours high</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Calendar (one developer)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Excel-ready (same as kitchen catalogue)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>150.0</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sheets with name, specs, embedded or folder images</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>18.0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>24.0</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>3–4 focused days</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Excel-ready (same as kitchen catalogue)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>180.0</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Sheets with name, specs, embedded or folder images</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>22.0</v>
+      </c>
+      <c r="E3" t="n">
+        <v>28.0</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>4–5 focused days</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Typical mixed cleanup</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>150.0</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Excel plus missing/wrong photos, spec label fixes</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>26.0</v>
+      </c>
+      <c r="E4" t="n">
+        <v>34.0</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>about 1–1.5 weeks</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Typical mixed cleanup</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>180.0</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Excel plus missing/wrong photos, spec label fixes</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>30.0</v>
+      </c>
+      <c r="E5" t="n">
+        <v>40.0</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>about 1.5–2 weeks</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Manual / messy source</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>150–180</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>PDFs, emails, uncropped photos — typed by hand</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>40.0</v>
+      </c>
+      <c r="E6" t="n">
+        <v>50.0</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2–3 weeks</t>
         </is>
       </c>
     </row>

</xml_diff>